<commit_message>
Daily slate 2026-06-01 [auto]
</commit_message>
<xml_diff>
--- a/ui_runner/templates/graded_analysis_tabs_2026-05-30.xlsx
+++ b/ui_runner/templates/graded_analysis_tabs_2026-05-30.xlsx
@@ -471,16 +471,16 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>191</v>
+        <v>196</v>
       </c>
       <c r="E2" t="n">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="F2" t="n">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="G2" t="n">
-        <v>42.4</v>
+        <v>43.4</v>
       </c>
     </row>
     <row r="3">
@@ -500,16 +500,16 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>188</v>
+        <v>195</v>
       </c>
       <c r="E3" t="n">
+        <v>98</v>
+      </c>
+      <c r="F3" t="n">
         <v>97</v>
       </c>
-      <c r="F3" t="n">
-        <v>91</v>
-      </c>
       <c r="G3" t="n">
-        <v>51.6</v>
+        <v>50.3</v>
       </c>
     </row>
     <row r="4">
@@ -529,16 +529,16 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="E4" t="n">
         <v>35</v>
       </c>
       <c r="F4" t="n">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="G4" t="n">
-        <v>44.3</v>
+        <v>43.2</v>
       </c>
     </row>
     <row r="5">
@@ -558,16 +558,16 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>116</v>
+        <v>125</v>
       </c>
       <c r="E5" t="n">
-        <v>55</v>
+        <v>61</v>
       </c>
       <c r="F5" t="n">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="G5" t="n">
-        <v>47.4</v>
+        <v>48.8</v>
       </c>
     </row>
     <row r="6">
@@ -587,16 +587,16 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>77</v>
+        <v>84</v>
       </c>
       <c r="E6" t="n">
-        <v>45</v>
+        <v>52</v>
       </c>
       <c r="F6" t="n">
         <v>32</v>
       </c>
       <c r="G6" t="n">
-        <v>58.4</v>
+        <v>61.9</v>
       </c>
     </row>
     <row r="7">
@@ -616,16 +616,16 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="E7" t="n">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="F7" t="n">
         <v>13</v>
       </c>
       <c r="G7" t="n">
-        <v>53.6</v>
+        <v>56.7</v>
       </c>
     </row>
     <row r="8">
@@ -645,16 +645,16 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>487</v>
+        <v>506</v>
       </c>
       <c r="E8" t="n">
-        <v>146</v>
+        <v>154</v>
       </c>
       <c r="F8" t="n">
-        <v>341</v>
+        <v>352</v>
       </c>
       <c r="G8" t="n">
-        <v>30</v>
+        <v>30.4</v>
       </c>
     </row>
     <row r="9">
@@ -703,16 +703,16 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>218</v>
+        <v>223</v>
       </c>
       <c r="E10" t="n">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="F10" t="n">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="G10" t="n">
-        <v>70.2</v>
+        <v>70.40000000000001</v>
       </c>
     </row>
     <row r="11">
@@ -732,16 +732,16 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>1045</v>
+        <v>1110</v>
       </c>
       <c r="E11" t="n">
-        <v>687</v>
+        <v>725</v>
       </c>
       <c r="F11" t="n">
-        <v>358</v>
+        <v>385</v>
       </c>
       <c r="G11" t="n">
-        <v>65.7</v>
+        <v>65.3</v>
       </c>
     </row>
     <row r="12">
@@ -761,16 +761,16 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>225</v>
+        <v>232</v>
       </c>
       <c r="E12" t="n">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="F12" t="n">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="G12" t="n">
-        <v>70.2</v>
+        <v>69.40000000000001</v>
       </c>
     </row>
     <row r="13">
@@ -790,16 +790,16 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>404</v>
+        <v>406</v>
       </c>
       <c r="E13" t="n">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="F13" t="n">
         <v>180</v>
       </c>
       <c r="G13" t="n">
-        <v>55.4</v>
+        <v>55.7</v>
       </c>
     </row>
     <row r="14">
@@ -819,16 +819,16 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>312</v>
+        <v>335</v>
       </c>
       <c r="E14" t="n">
-        <v>93</v>
+        <v>103</v>
       </c>
       <c r="F14" t="n">
-        <v>219</v>
+        <v>232</v>
       </c>
       <c r="G14" t="n">
-        <v>29.8</v>
+        <v>30.7</v>
       </c>
     </row>
     <row r="15">
@@ -848,16 +848,16 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>412</v>
+        <v>447</v>
       </c>
       <c r="E15" t="n">
-        <v>69</v>
+        <v>80</v>
       </c>
       <c r="F15" t="n">
-        <v>343</v>
+        <v>367</v>
       </c>
       <c r="G15" t="n">
-        <v>16.7</v>
+        <v>17.9</v>
       </c>
     </row>
     <row r="16">
@@ -877,16 +877,16 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>141</v>
+        <v>147</v>
       </c>
       <c r="E16" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F16" t="n">
-        <v>122</v>
+        <v>127</v>
       </c>
       <c r="G16" t="n">
-        <v>13.5</v>
+        <v>13.6</v>
       </c>
     </row>
     <row r="17">
@@ -906,13 +906,13 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>4837</v>
+        <v>5134</v>
       </c>
       <c r="E17" t="n">
-        <v>1222</v>
+        <v>1299</v>
       </c>
       <c r="F17" t="n">
-        <v>3615</v>
+        <v>3835</v>
       </c>
       <c r="G17" t="n">
         <v>25.3</v>
@@ -1106,49 +1106,52 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>82.09999999999999</v>
+        <v>82.8</v>
       </c>
       <c r="C2" t="n">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="D2" t="n">
-        <v>93.59999999999999</v>
+        <v>93.8</v>
       </c>
       <c r="E2" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="F2" t="n">
-        <v>80.59999999999999</v>
+        <v>78.8</v>
       </c>
       <c r="G2" t="n">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="H2" t="n">
-        <v>53.8</v>
+        <v>54.4</v>
       </c>
       <c r="I2" t="n">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="J2" t="n">
         <v>100</v>
       </c>
       <c r="K2" t="n">
-        <v>1</v>
+        <v>3</v>
+      </c>
+      <c r="L2" t="n">
+        <v>41.7</v>
       </c>
       <c r="M2" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="N2" t="n">
-        <v>33.3</v>
+        <v>40</v>
       </c>
       <c r="O2" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="P2" t="n">
-        <v>23.4</v>
+        <v>23.5</v>
       </c>
       <c r="Q2" t="n">
-        <v>316</v>
+        <v>319</v>
       </c>
       <c r="R2" t="n">
         <v>33.3</v>
@@ -1169,16 +1172,16 @@
         <v>1</v>
       </c>
       <c r="X2" t="n">
-        <v>35.1</v>
+        <v>35.3</v>
       </c>
       <c r="Y2" t="n">
-        <v>259</v>
+        <v>269</v>
       </c>
       <c r="Z2" t="n">
-        <v>60</v>
+        <v>27.3</v>
       </c>
       <c r="AA2" t="n">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="AB2" t="n">
         <v>46.2</v>
@@ -1376,22 +1379,22 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>57.1</v>
+        <v>60</v>
       </c>
       <c r="C5" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="D5" t="n">
-        <v>28.6</v>
+        <v>33.3</v>
       </c>
       <c r="E5" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F5" t="n">
-        <v>11.1</v>
+        <v>18.2</v>
       </c>
       <c r="G5" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="H5" t="n">
         <v>0</v>
@@ -1403,25 +1406,25 @@
         <v>0</v>
       </c>
       <c r="K5" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="L5" t="n">
-        <v>10.3</v>
+        <v>16.2</v>
       </c>
       <c r="M5" t="n">
-        <v>29</v>
+        <v>37</v>
       </c>
       <c r="N5" t="n">
         <v>0</v>
       </c>
       <c r="O5" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="P5" t="n">
-        <v>0</v>
+        <v>6.7</v>
       </c>
       <c r="Q5" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="R5" t="n">
         <v>50</v>
@@ -1436,16 +1439,16 @@
         <v>0</v>
       </c>
       <c r="X5" t="n">
-        <v>20</v>
+        <v>29.2</v>
       </c>
       <c r="Y5" t="n">
-        <v>15</v>
+        <v>24</v>
       </c>
       <c r="Z5" t="n">
-        <v>78.8</v>
+        <v>79.40000000000001</v>
       </c>
       <c r="AA5" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="AB5" t="n">
         <v>100</v>
@@ -1558,94 +1561,94 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>70.2</v>
+        <v>70.40000000000001</v>
       </c>
       <c r="C7" t="n">
-        <v>218</v>
+        <v>223</v>
       </c>
       <c r="D7" t="n">
-        <v>65.7</v>
+        <v>65.3</v>
       </c>
       <c r="E7" t="n">
-        <v>1045</v>
+        <v>1110</v>
       </c>
       <c r="F7" t="n">
-        <v>70.2</v>
+        <v>69.40000000000001</v>
       </c>
       <c r="G7" t="n">
-        <v>225</v>
+        <v>232</v>
       </c>
       <c r="H7" t="n">
-        <v>55.4</v>
+        <v>55.7</v>
       </c>
       <c r="I7" t="n">
-        <v>404</v>
+        <v>406</v>
       </c>
       <c r="J7" t="n">
-        <v>29.8</v>
+        <v>30.7</v>
       </c>
       <c r="K7" t="n">
-        <v>312</v>
+        <v>335</v>
       </c>
       <c r="L7" t="n">
-        <v>16.7</v>
+        <v>17.9</v>
       </c>
       <c r="M7" t="n">
-        <v>412</v>
+        <v>447</v>
       </c>
       <c r="N7" t="n">
-        <v>13.5</v>
+        <v>13.6</v>
       </c>
       <c r="O7" t="n">
-        <v>141</v>
+        <v>147</v>
       </c>
       <c r="P7" t="n">
         <v>25.3</v>
       </c>
       <c r="Q7" t="n">
-        <v>4837</v>
+        <v>5134</v>
       </c>
       <c r="R7" t="n">
-        <v>42.4</v>
+        <v>43.4</v>
       </c>
       <c r="S7" t="n">
-        <v>191</v>
+        <v>196</v>
       </c>
       <c r="T7" t="n">
-        <v>44.3</v>
+        <v>43.2</v>
       </c>
       <c r="U7" t="n">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="V7" t="n">
-        <v>58.4</v>
+        <v>61.9</v>
       </c>
       <c r="W7" t="n">
-        <v>77</v>
+        <v>84</v>
       </c>
       <c r="X7" t="n">
+        <v>30.4</v>
+      </c>
+      <c r="Y7" t="n">
+        <v>506</v>
+      </c>
+      <c r="Z7" t="n">
+        <v>50.3</v>
+      </c>
+      <c r="AA7" t="n">
+        <v>195</v>
+      </c>
+      <c r="AB7" t="n">
+        <v>48.8</v>
+      </c>
+      <c r="AC7" t="n">
+        <v>125</v>
+      </c>
+      <c r="AD7" t="n">
+        <v>56.7</v>
+      </c>
+      <c r="AE7" t="n">
         <v>30</v>
-      </c>
-      <c r="Y7" t="n">
-        <v>487</v>
-      </c>
-      <c r="Z7" t="n">
-        <v>51.6</v>
-      </c>
-      <c r="AA7" t="n">
-        <v>188</v>
-      </c>
-      <c r="AB7" t="n">
-        <v>47.4</v>
-      </c>
-      <c r="AC7" t="n">
-        <v>116</v>
-      </c>
-      <c r="AD7" t="n">
-        <v>53.6</v>
-      </c>
-      <c r="AE7" t="n">
-        <v>28</v>
       </c>
       <c r="AF7" t="n">
         <v>66.3</v>

</xml_diff>